<commit_message>
chore: catch-up + gitignore cleanup + 3 fixes (B, C, E)
</commit_message>
<xml_diff>
--- a/Causas con liq/Causas_con_liquidacion.xlsx
+++ b/Causas con liq/Causas_con_liquidacion.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excedentes Confirmados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revision Manual" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,61 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
-        <bgColor rgb="00D6E4F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
-        <bgColor rgb="00ED7D31"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -88,41 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <bottom style="thick">
-        <color rgb="001F4E79"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,211 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
-          <t>Causa (ROL)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Tribunal</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Demandado</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Direccion</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Comuna</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Deuda Original ($)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Precio Remate ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Deuda Liquidada ($)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Excedente Confirmado ($)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha Remate</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>LIQUIDACIONES ENCONTRADAS EL 02/04/2026 (1 nuevas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>C-1529-2023</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>3º Juzgado Civil de Temuco</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>CRISTIAN ANDRÉS FARÍAS LUCERO</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Andalué número mil cuatrocientos cuarenta, sector Andalué, Condominio Atalaya de Andalué</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>San Pedro de la Paz</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>52019470</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>131700791</v>
-      </c>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="5" t="n">
-        <v>61986279</v>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>EXCEDENTE_CONFIRMADO</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:K2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Causa (ROL)</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Tribunal</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Demandado</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>Direccion</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>Comuna</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Deuda Original ($)</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>Precio Remate ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>Credito Adeudado ($)</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>Fecha Remate</t>
-        </is>
-      </c>
-      <c r="J1" s="6" t="inlineStr">
-        <is>
-          <t>Estado</t>
+          <t>No hay excedentes confirmados</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: actualizar Excel madre + historial + BD interna (estado post fix OCR de actas)
Causas_posible_saldo.xlsx, causas_eliminadas_historial.csv,
Causas_con_liquidacion.xlsx y causas_ojv.xlsx reflejan el estado real
tras el ciclo Audit6.1 (fix OCR de actas + reproceso).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Causas con liq/Causas_con_liquidacion.xlsx
+++ b/Causas con liq/Causas_con_liquidacion.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,55 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -42,12 +81,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <bottom style="thick">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,17 +478,137 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No hay excedentes confirmados</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Causa (ROL)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tribunal</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Demandado</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Direccion</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Comuna</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Deuda Original ($)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Precio Remate ($)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Deuda Liquidada ($)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Excedente Confirmado ($)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fecha Remate</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LIQUIDACIONES ENCONTRADAS EL 23/05/2026 (1 nuevas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>C-2100-2024</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2º Juzgado Civil de Valparaíso</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>EUGENIO BENJAMÍN MELLA RIVAS</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Las Maravillas número 201</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Viña del Mar</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>7043345</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>27691792</v>
+      </c>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="5" t="n">
+        <v>365499</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>EXCEDENTE_CONFIRMADO</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:K2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>